<commit_message>
refactor: Improve episode date handling in condition aggregation and optimize imports in message router
</commit_message>
<xml_diff>
--- a/backend/tests/DB_Tables_Report.xlsx
+++ b/backend/tests/DB_Tables_Report.xlsx
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -613,12 +613,12 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>13/1/23</t>
+          <t>2023-01-13</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>13/1/23</t>
+          <t>2023-01-13</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -630,7 +630,7 @@
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>Metrogyl 200 [1 tab] once daily end=None dur=5d | Digene [1 tab] once daily end=None dur=10d | Nutrolin B [1 cap] once daily end=None dur=10d</t>
+          <t>Metronidazole [200 mg] Once daily end=None dur=5d | Digene [None] Once daily end=None dur=10d | Nutracillin B13 [None] Once daily end=None dur=10d</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr"/>
@@ -714,7 +714,7 @@
       <c r="J7" s="3" t="inlineStr"/>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>Onyfle lotion [None] Twice daily end=None dur=10d</t>
+          <t>Onfite lotion [None] Twice daily end=None dur=10d</t>
         </is>
       </c>
       <c r="L7" s="3" t="inlineStr"/>
@@ -754,7 +754,7 @@
       <c r="J8" s="2" t="inlineStr"/>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Onyfle lotion [None] Twice daily end=None dur=10d</t>
+          <t>Nuforce Pet 200 [1 tablet] Once daily end=None dur=10d</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr"/>
@@ -762,15 +762,15 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>4cc61ecc-8ab9-4348-9905-a710c3c0e65a.JPG</t>
+          <t>887afa02-5a78-4725-8c70-3e1c81ec7ded.JPG</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Ear mites (inferred)</t>
+          <t>Post-neuter surgical care</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -783,22 +783,42 @@
           <t>active</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr"/>
-      <c r="G9" s="3" t="inlineStr"/>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>31/1/23</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>31/1/23</t>
+        </is>
+      </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
           <t>inferred</t>
         </is>
       </c>
-      <c r="I9" s="3" t="n"/>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>Post-operative care following neutering under general anesthesia.</t>
+        </is>
+      </c>
       <c r="J9" s="3" t="inlineStr"/>
-      <c r="K9" s="3" t="inlineStr"/>
-      <c r="L9" s="3" t="inlineStr"/>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>Rivcet spray [None] Twice daily end=None dur=10d | Wound Heal powder [None] Once daily end=None dur=10d | Capril 100 [None] Once daily end=None dur=10d | Cefpet CLV [None] Once daily end=None dur=10d | Pantopet 40 [None] Once daily end=None dur=10d</t>
+        </is>
+      </c>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>Recheck recheck=8/2/23 | Recheck recheck=13/2/23</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>887afa02-5a78-4725-8c70-3e1c81ec7ded.JPG</t>
+          <t>cb8881ad-2432-49f8-91a4-3aa752b4d4a1.JPG</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -806,7 +826,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Post-neuter care (inferred)</t>
+          <t>Musculoskeletal pain (inferred)</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -821,12 +841,12 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>31/1/23</t>
+          <t>05/12/2022</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>31/1/23</t>
+          <t>05/12/2022</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -834,22 +854,14 @@
           <t>inferred</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>Post-surgical care following neutering under general anesthesia.</t>
-        </is>
-      </c>
+      <c r="I10" s="2" t="n"/>
       <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Riovet spray [None] Twice daily end=None dur=10d | Wound Heal powder [None] Once daily end=None dur=10d | Caprill 100 [None] Once daily end=None dur=10d | Cefpet CV [None] Once daily end=None dur=10d | Pantopet 40 [None] Once daily end=None dur=10d</t>
-        </is>
-      </c>
-      <c r="L10" s="2" t="inlineStr">
-        <is>
-          <t>Recheck recheck=8/2/23 | Recheck recheck=13/2/23</t>
-        </is>
-      </c>
+          <t>Carital [10 mg, 1/2 tablet] once daily end=None dur=5d</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -858,7 +870,7 @@
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
@@ -894,7 +906,7 @@
       <c r="J11" s="3" t="inlineStr"/>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>Cartail 10mg [1/2 tab] once daily end=None dur=5d</t>
+          <t>Hot fomentation [None] None end=None dur=Noned</t>
         </is>
       </c>
       <c r="L11" s="3" t="inlineStr"/>
@@ -902,124 +914,76 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>cb8881ad-2432-49f8-91a4-3aa752b4d4a1.JPG</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="n">
-        <v>2</v>
-      </c>
+          <t>df197d05-b771-4de0-8b16-236a96bbdf7a.JPG</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr"/>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Musculoskeletal pain (inferred)</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>episodic</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>05/12/2022</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>05/12/2022</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>inferred</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="n"/>
+          <t>(no conditions extracted)</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr"/>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>Hot fomentation [None] None end=None dur=Noned</t>
-        </is>
-      </c>
+      <c r="K12" s="2" t="inlineStr"/>
       <c r="L12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>df197d05-b771-4de0-8b16-236a96bbdf7a.JPG</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr"/>
+          <t>f4d47d0c-db22-43c6-b757-9b10adb74446.JPG</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>(no conditions extracted)</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr"/>
-      <c r="E13" s="3" t="inlineStr"/>
-      <c r="F13" s="3" t="inlineStr"/>
-      <c r="G13" s="3" t="inlineStr"/>
-      <c r="H13" s="3" t="inlineStr"/>
-      <c r="I13" s="3" t="inlineStr"/>
+          <t>Pyoderma</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>episodic</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>2024-12-19</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>2024-12-19</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>Skin infection with pyoderma and fungal infection.</t>
+        </is>
+      </c>
       <c r="J13" s="3" t="inlineStr"/>
-      <c r="K13" s="3" t="inlineStr"/>
-      <c r="L13" s="3" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>f4d47d0c-db22-43c6-b757-9b10adb74446.JPG</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Pyoderma</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>episodic</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>2024-12-19</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>2024-12-19</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>explicit</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>Pyoderma diagnosed based on clinical findings.</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr"/>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>Itavet [None] None end=None dur=10d | Panchbat D [None] None end=None dur=10d | Onfyte lotion [None] Twice daily end=None dur=10d</t>
-        </is>
-      </c>
-      <c r="L14" s="2" t="inlineStr">
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>Itraconazole [None] None end=None dur=10d | Pantoprazole+Domperidone [None] None end=None dur=10d | Onfyte lotion [None] Twice daily end=None dur=10d</t>
+        </is>
+      </c>
+      <c r="L13" s="3" t="inlineStr">
         <is>
           <t>Recheck recheck=None</t>
         </is>
@@ -1036,7 +1000,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1322,7 +1286,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>c_doc_4cc61ecc-8ab9-4348-9905-a710c3c0e65a_JPG_2</t>
+          <t>c_doc_887afa02-5a78-4725-8c70-3e1c81ec7ded_JPG_0</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -1332,12 +1296,12 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>doc_4cc61ecc-8ab9-4348-9905-a710c3c0e65a_JPG</t>
+          <t>doc_887afa02-5a78-4725-8c70-3e1c81ec7ded_JPG</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Ear mites (inferred)</t>
+          <t>Post-neuter surgical care</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -1350,9 +1314,21 @@
           <t>resolved</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr"/>
-      <c r="H5" s="3" t="inlineStr"/>
-      <c r="I5" s="3" t="inlineStr"/>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>2023-01-31</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>2023-01-31</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>2023-02-10</t>
+        </is>
+      </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
           <t>extraction</t>
@@ -1382,7 +1358,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>c_doc_887afa02-5a78-4725-8c70-3e1c81ec7ded_JPG_0</t>
+          <t>c_doc_cb8881ad-2432-49f8-91a4-3aa752b4d4a1_JPG_0</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -1392,12 +1368,12 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>doc_887afa02-5a78-4725-8c70-3e1c81ec7ded_JPG</t>
+          <t>doc_cb8881ad-2432-49f8-91a4-3aa752b4d4a1_JPG</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Post-neuter care (inferred)</t>
+          <t>Musculoskeletal pain (inferred)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -1412,17 +1388,17 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>2023-01-31</t>
+          <t>2022-12-05</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>2023-01-31</t>
+          <t>2022-12-05</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>2023-02-10</t>
+          <t>2022-12-10</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -1454,7 +1430,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>c_doc_cb8881ad-2432-49f8-91a4-3aa752b4d4a1_JPG_0</t>
+          <t>c_doc_f4d47d0c-db22-43c6-b757-9b10adb74446_JPG_0</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -1464,12 +1440,12 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>doc_cb8881ad-2432-49f8-91a4-3aa752b4d4a1_JPG</t>
+          <t>doc_f4d47d0c-db22-43c6-b757-9b10adb74446_JPG</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Musculoskeletal pain (inferred)</t>
+          <t>Pyoderma</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -1484,17 +1460,17 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>2022-12-05</t>
+          <t>2024-12-19</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>2022-12-05</t>
+          <t>2024-12-19</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>2022-12-10</t>
+          <t>2024-12-29</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
@@ -1518,78 +1494,6 @@
         </is>
       </c>
       <c r="N7" s="3" t="inlineStr">
-        <is>
-          <t>(set at insert)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>c_doc_f4d47d0c-db22-43c6-b757-9b10adb74446_JPG_0</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>test_pet</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>doc_f4d47d0c-db22-43c6-b757-9b10adb74446_JPG</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Pyoderma</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>episodic</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>resolved</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>2024-12-19</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>2024-12-19</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>2024-12-29</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>extraction</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="inlineStr">
-        <is>
-          <t>(set by aggregation)</t>
-        </is>
-      </c>
-      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>(set at insert)</t>
         </is>
@@ -1612,8 +1516,8 @@
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
     <col width="37" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
@@ -1691,12 +1595,12 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Metrogyl 200</t>
+          <t>Metronidazole</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>1 tab</t>
+          <t>200 mg</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr"/>
@@ -1734,11 +1638,7 @@
           <t>Digene</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>1 tab</t>
-        </is>
-      </c>
+      <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="3" t="inlineStr"/>
       <c r="G3" s="3" t="inlineStr"/>
       <c r="H3" s="3" t="inlineStr"/>
@@ -1771,14 +1671,10 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Nutrolin B</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>1 cap</t>
-        </is>
-      </c>
+          <t>Nutracillin B13</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr"/>
       <c r="G4" s="2" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1811,7 +1707,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Onyfle lotion</t>
+          <t>Onfite lotion</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr"/>
@@ -1843,10 +1739,14 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Onyfle lotion</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr"/>
+          <t>Nuforce Pet 200</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>1 tablet</t>
+        </is>
+      </c>
       <c r="F6" s="2" t="inlineStr"/>
       <c r="G6" s="2" t="inlineStr"/>
       <c r="H6" s="2" t="inlineStr"/>
@@ -1870,12 +1770,12 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Post-neuter care (inferred)</t>
+          <t>Post-neuter surgical care</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Riovet spray</t>
+          <t>Rivcet spray</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr"/>
@@ -1906,7 +1806,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Post-neuter care (inferred)</t>
+          <t>Post-neuter surgical care</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -1942,12 +1842,12 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Post-neuter care (inferred)</t>
+          <t>Post-neuter surgical care</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Caprill 100</t>
+          <t>Capril 100</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr"/>
@@ -1978,12 +1878,12 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Post-neuter care (inferred)</t>
+          <t>Post-neuter surgical care</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Cefpet CV</t>
+          <t>Cefpet CLV</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
@@ -2014,7 +1914,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Post-neuter care (inferred)</t>
+          <t>Post-neuter surgical care</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -2055,12 +1955,12 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Cartail 10mg</t>
+          <t>Carital</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>1/2 tab</t>
+          <t>10 mg, 1/2 tablet</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr"/>
@@ -2127,7 +2027,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Itavet</t>
+          <t>Itraconazole</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
@@ -2163,7 +2063,7 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Panchbat D</t>
+          <t>Pantoprazole+Domperidone</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr"/>
@@ -2233,7 +2133,7 @@
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="29" customWidth="1" min="3" max="3"/>
+    <col width="27" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
@@ -2284,7 +2184,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Post-neuter care (inferred)</t>
+          <t>Post-neuter surgical care</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -2312,7 +2212,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Post-neuter care (inferred)</t>
+          <t>Post-neuter surgical care</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -2362,7 +2262,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2370,7 +2270,7 @@
     <col width="37" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="21" customWidth="1" min="9" max="9"/>
@@ -2530,7 +2430,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>episodic</t>
+          <t>recurrent</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -2540,17 +2440,17 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
+          <t>2024-12-19, 2026-05-01, 2026-05-02</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
           <t>2024-12-19</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>2024-12-19</t>
-        </is>
-      </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>2024-12-19</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -2560,12 +2460,12 @@
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="L3" s="3" t="inlineStr">
@@ -2590,7 +2490,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Ear mites (inferred)</t>
+          <t>Post-neuter surgical care</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -2603,13 +2503,29 @@
           <t>resolved</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>2023-01-31</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>2023-01-31</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>2023-01-31</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>2023-02-10</t>
+        </is>
+      </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -2619,7 +2535,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>c_doc_4cc61ecc-8ab9-4348-9905-a710c3c0e65a_JPG_2</t>
+          <t>c_doc_887afa02-5a78-4725-8c70-3e1c81ec7ded_JPG_0</t>
         </is>
       </c>
       <c r="M4" s="2" t="n">
@@ -2639,7 +2555,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Post-neuter care (inferred)</t>
+          <t>Musculoskeletal pain (inferred)</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -2654,22 +2570,22 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>2023-01-31</t>
+          <t>2022-12-05</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>2023-01-31</t>
+          <t>2022-12-05</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>2023-01-31</t>
+          <t>2022-12-05</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>2023-02-10</t>
+          <t>2022-12-10</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
@@ -2684,75 +2600,10 @@
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>c_doc_887afa02-5a78-4725-8c70-3e1c81ec7ded_JPG_0</t>
+          <t>c_doc_cb8881ad-2432-49f8-91a4-3aa752b4d4a1_JPG_0</t>
         </is>
       </c>
       <c r="M5" s="3" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>(uuid — set at upsert)</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>test_pet</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Musculoskeletal pain (inferred)</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>episodic</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>resolved</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>2022-12-05</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>2022-12-05</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>2022-12-05</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>2022-12-10</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>c_doc_cb8881ad-2432-49f8-91a4-3aa752b4d4a1_JPG_0</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2767,13 +2618,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="37" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -2812,7 +2663,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Metrogyl 200</t>
+          <t>Metronidazole</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -2822,7 +2673,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>1 tab</t>
+          <t>200 mg</t>
         </is>
       </c>
       <c r="E2" s="2" t="n"/>
@@ -2843,11 +2694,7 @@
           <t>2023-01-23</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>1 tab</t>
-        </is>
-      </c>
+      <c r="D3" s="3" t="n"/>
       <c r="E3" s="3" t="n"/>
     </row>
     <row r="4">
@@ -2858,7 +2705,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Nutrolin B</t>
+          <t>Nutracillin B13</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -2866,11 +2713,7 @@
           <t>2023-01-23</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>1 cap</t>
-        </is>
-      </c>
+      <c r="D4" s="2" t="n"/>
       <c r="E4" s="2" t="n"/>
     </row>
     <row r="5">
@@ -2881,7 +2724,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Onyfle lotion</t>
+          <t>Onfite lotion</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr"/>
@@ -2896,15 +2739,15 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Itavet</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>2024-12-29</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="n"/>
+          <t>Nuforce Pet 200</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr"/>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>1 tablet</t>
+        </is>
+      </c>
       <c r="E6" s="2" t="n"/>
     </row>
     <row r="7">
@@ -2915,7 +2758,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Panchbat D</t>
+          <t>Itraconazole</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -2934,7 +2777,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Onfyte lotion</t>
+          <t>Pantoprazole+Domperidone</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -2948,17 +2791,17 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Post-neuter care (inferred)</t>
+          <t>Pyoderma (inferred)</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Riovet spray</t>
+          <t>Onfyte lotion</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>2023-02-10</t>
+          <t>2024-12-29</t>
         </is>
       </c>
       <c r="D9" s="3" t="n"/>
@@ -2967,12 +2810,12 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Post-neuter care (inferred)</t>
+          <t>Post-neuter surgical care</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Wound Heal powder</t>
+          <t>Rivcet spray</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -2986,12 +2829,12 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Post-neuter care (inferred)</t>
+          <t>Post-neuter surgical care</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Caprill 100</t>
+          <t>Wound Heal powder</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -3005,12 +2848,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Post-neuter care (inferred)</t>
+          <t>Post-neuter surgical care</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Cefpet CV</t>
+          <t>Capril 100</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -3024,12 +2867,12 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Post-neuter care (inferred)</t>
+          <t>Post-neuter surgical care</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Pantopet 40</t>
+          <t>Cefpet CLV</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -3043,24 +2886,20 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Musculoskeletal pain (inferred)</t>
+          <t>Post-neuter surgical care</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Cartail 10mg</t>
+          <t>Pantopet 40</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>2022-12-10</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>1/2 tab</t>
-        </is>
-      </c>
+          <t>2023-02-10</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="n"/>
       <c r="E14" s="2" t="n"/>
     </row>
     <row r="15">
@@ -3071,12 +2910,35 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
+          <t>Carital</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>2022-12-10</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>10 mg, 1/2 tablet</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Musculoskeletal pain (inferred)</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
           <t>Hot fomentation</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr"/>
-      <c r="D15" s="3" t="n"/>
-      <c r="E15" s="3" t="n"/>
+      <c r="C16" s="2" t="inlineStr"/>
+      <c r="D16" s="2" t="n"/>
+      <c r="E16" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: Allow 'inferred' as a valid condition source and update related logic in condition handling
</commit_message>
<xml_diff>
--- a/backend/tests/DB_Tables_Report.xlsx
+++ b/backend/tests/DB_Tables_Report.xlsx
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -630,7 +630,7 @@
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>Metronidazole [200 mg] Once daily end=None dur=5d | Digene [None] Once daily end=None dur=10d | Nutracillin B13 [None] Once daily end=None dur=10d</t>
+          <t>Metronidazole [200 mg] Once daily end=None dur=5d | Digene [None] Once daily end=None dur=10d | Nutrolin B [None] Once daily end=None dur=10d</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr"/>
@@ -690,7 +690,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Pyoderma (inferred)</t>
+          <t>Pyoderma</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -707,14 +707,14 @@
       <c r="G7" s="3" t="inlineStr"/>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>inferred</t>
+          <t>explicit</t>
         </is>
       </c>
       <c r="I7" s="3" t="n"/>
       <c r="J7" s="3" t="inlineStr"/>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>Onfite lotion [None] Twice daily end=None dur=10d</t>
+          <t>Betadine [None] Twice daily end=None dur=10d | Onyfle lotion [None] Twice daily end=None dur=10d | Nuforce Pet 200 [1 tablet] Once daily end=None dur=10d</t>
         </is>
       </c>
       <c r="L7" s="3" t="inlineStr"/>
@@ -722,15 +722,15 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>4cc61ecc-8ab9-4348-9905-a710c3c0e65a.JPG</t>
+          <t>887afa02-5a78-4725-8c70-3e1c81ec7ded.JPG</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Fungal infection (inferred)</t>
+          <t>Post-neutering care (inferred)</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -743,26 +743,42 @@
           <t>active</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr"/>
-      <c r="G8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>31/1/23</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>31/1/23</t>
+        </is>
+      </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
           <t>inferred</t>
         </is>
       </c>
-      <c r="I8" s="2" t="n"/>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Post-surgical care following neutering under general anesthesia.</t>
+        </is>
+      </c>
       <c r="J8" s="2" t="inlineStr"/>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Nuforce Pet 200 [1 tablet] Once daily end=None dur=10d</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr"/>
+          <t>Rivcet spray [None] Twice daily end=None dur=10d | Wound Heal powder [None] Once daily end=None dur=10d | Capril 100 [None] Once daily end=None dur=10d | Cefpet-CLV [None] Once daily end=None dur=10d | Pantopet 40 [None] Once daily end=None dur=10d</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Recheck recheck=8/2/23 | Recheck recheck=13/2/23</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>887afa02-5a78-4725-8c70-3e1c81ec7ded.JPG</t>
+          <t>cb8881ad-2432-49f8-91a4-3aa752b4d4a1.JPG</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
@@ -770,7 +786,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Post-neuter surgical care</t>
+          <t>Musculoskeletal pain (inferred)</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -785,12 +801,12 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>31/1/23</t>
+          <t>05/12/2022</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>31/1/23</t>
+          <t>05/12/2022</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
@@ -798,22 +814,14 @@
           <t>inferred</t>
         </is>
       </c>
-      <c r="I9" s="3" t="inlineStr">
-        <is>
-          <t>Post-operative care following neutering under general anesthesia.</t>
-        </is>
-      </c>
+      <c r="I9" s="3" t="n"/>
       <c r="J9" s="3" t="inlineStr"/>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>Rivcet spray [None] Twice daily end=None dur=10d | Wound Heal powder [None] Once daily end=None dur=10d | Capril 100 [None] Once daily end=None dur=10d | Cefpet CLV [None] Once daily end=None dur=10d | Pantopet 40 [None] Once daily end=None dur=10d</t>
-        </is>
-      </c>
-      <c r="L9" s="3" t="inlineStr">
-        <is>
-          <t>Recheck recheck=8/2/23 | Recheck recheck=13/2/23</t>
-        </is>
-      </c>
+          <t>Carital [10 mg, 1/2 tablet] once daily end=None dur=5d</t>
+        </is>
+      </c>
+      <c r="L9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -822,7 +830,7 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -854,136 +862,88 @@
           <t>inferred</t>
         </is>
       </c>
-      <c r="I10" s="2" t="n"/>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Hot fomentation advised</t>
+        </is>
+      </c>
       <c r="J10" s="2" t="inlineStr"/>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>Carital [10 mg, 1/2 tablet] once daily end=None dur=5d</t>
-        </is>
-      </c>
+      <c r="K10" s="2" t="inlineStr"/>
       <c r="L10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>cb8881ad-2432-49f8-91a4-3aa752b4d4a1.JPG</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="n">
-        <v>2</v>
-      </c>
+          <t>df197d05-b771-4de0-8b16-236a96bbdf7a.JPG</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr"/>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Musculoskeletal pain (inferred)</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>episodic</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>05/12/2022</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>05/12/2022</t>
-        </is>
-      </c>
-      <c r="H11" s="3" t="inlineStr">
-        <is>
-          <t>inferred</t>
-        </is>
-      </c>
-      <c r="I11" s="3" t="n"/>
+          <t>(no conditions extracted)</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr"/>
+      <c r="F11" s="3" t="inlineStr"/>
+      <c r="G11" s="3" t="inlineStr"/>
+      <c r="H11" s="3" t="inlineStr"/>
+      <c r="I11" s="3" t="inlineStr"/>
       <c r="J11" s="3" t="inlineStr"/>
-      <c r="K11" s="3" t="inlineStr">
-        <is>
-          <t>Hot fomentation [None] None end=None dur=Noned</t>
-        </is>
-      </c>
+      <c r="K11" s="3" t="inlineStr"/>
       <c r="L11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>df197d05-b771-4de0-8b16-236a96bbdf7a.JPG</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr"/>
+          <t>f4d47d0c-db22-43c6-b757-9b10adb74446.JPG</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>(no conditions extracted)</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr"/>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr"/>
-      <c r="I12" s="2" t="inlineStr"/>
+          <t>Pyoderma</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>episodic</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>2024-12-19</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>2024-12-19</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Bacterial skin infection (pyoderma) diagnosed based on clinical findings.</t>
+        </is>
+      </c>
       <c r="J12" s="2" t="inlineStr"/>
-      <c r="K12" s="2" t="inlineStr"/>
-      <c r="L12" s="2" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>f4d47d0c-db22-43c6-b757-9b10adb74446.JPG</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>Pyoderma</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>episodic</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>2024-12-19</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>2024-12-19</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="inlineStr">
-        <is>
-          <t>explicit</t>
-        </is>
-      </c>
-      <c r="I13" s="3" t="inlineStr">
-        <is>
-          <t>Skin infection with pyoderma and fungal infection.</t>
-        </is>
-      </c>
-      <c r="J13" s="3" t="inlineStr"/>
-      <c r="K13" s="3" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>Itraconazole [None] None end=None dur=10d | Pantoprazole+Domperidone [None] None end=None dur=10d | Onfyte lotion [None] Twice daily end=None dur=10d</t>
         </is>
       </c>
-      <c r="L13" s="3" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>Recheck recheck=None</t>
         </is>
@@ -1000,7 +960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1181,7 +1141,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Pyoderma (inferred)</t>
+          <t>Pyoderma</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -1226,7 +1186,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>c_doc_4cc61ecc-8ab9-4348-9905-a710c3c0e65a_JPG_1</t>
+          <t>c_doc_887afa02-5a78-4725-8c70-3e1c81ec7ded_JPG_0</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -1236,12 +1196,12 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>doc_4cc61ecc-8ab9-4348-9905-a710c3c0e65a_JPG</t>
+          <t>doc_887afa02-5a78-4725-8c70-3e1c81ec7ded_JPG</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Fungal infection (inferred)</t>
+          <t>Post-neutering care (inferred)</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -1254,9 +1214,21 @@
           <t>resolved</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>2023-01-31</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>2023-01-31</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>2023-02-10</t>
+        </is>
+      </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
           <t>extraction</t>
@@ -1286,7 +1258,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>c_doc_887afa02-5a78-4725-8c70-3e1c81ec7ded_JPG_0</t>
+          <t>c_doc_cb8881ad-2432-49f8-91a4-3aa752b4d4a1_JPG_0</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -1296,12 +1268,12 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>doc_887afa02-5a78-4725-8c70-3e1c81ec7ded_JPG</t>
+          <t>doc_cb8881ad-2432-49f8-91a4-3aa752b4d4a1_JPG</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Post-neuter surgical care</t>
+          <t>Musculoskeletal pain (inferred)</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -1316,17 +1288,17 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>2023-01-31</t>
+          <t>2022-12-05</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>2023-01-31</t>
+          <t>2022-12-05</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>2023-02-10</t>
+          <t>2022-12-10</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
@@ -1358,7 +1330,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>c_doc_cb8881ad-2432-49f8-91a4-3aa752b4d4a1_JPG_0</t>
+          <t>c_doc_f4d47d0c-db22-43c6-b757-9b10adb74446_JPG_0</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -1368,12 +1340,12 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>doc_cb8881ad-2432-49f8-91a4-3aa752b4d4a1_JPG</t>
+          <t>doc_f4d47d0c-db22-43c6-b757-9b10adb74446_JPG</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Musculoskeletal pain (inferred)</t>
+          <t>Pyoderma</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -1388,17 +1360,17 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>2022-12-05</t>
+          <t>2024-12-19</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>2022-12-05</t>
+          <t>2024-12-19</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>2022-12-10</t>
+          <t>2024-12-29</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -1422,78 +1394,6 @@
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
-        <is>
-          <t>(set at insert)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>c_doc_f4d47d0c-db22-43c6-b757-9b10adb74446_JPG_0</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>test_pet</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>doc_f4d47d0c-db22-43c6-b757-9b10adb74446_JPG</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>Pyoderma</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>episodic</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>resolved</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>2024-12-19</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>2024-12-19</t>
-        </is>
-      </c>
-      <c r="I7" s="3" t="inlineStr">
-        <is>
-          <t>2024-12-29</t>
-        </is>
-      </c>
-      <c r="J7" s="3" t="inlineStr">
-        <is>
-          <t>extraction</t>
-        </is>
-      </c>
-      <c r="K7" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="L7" s="3" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="M7" s="3" t="inlineStr">
-        <is>
-          <t>(set by aggregation)</t>
-        </is>
-      </c>
-      <c r="N7" s="3" t="inlineStr">
         <is>
           <t>(set at insert)</t>
         </is>
@@ -1671,7 +1571,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Nutracillin B13</t>
+          <t>Nutrolin B</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
@@ -1702,12 +1602,12 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Pyoderma (inferred)</t>
+          <t>Pyoderma</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Onfite lotion</t>
+          <t>Betadine</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr"/>
@@ -1729,24 +1629,20 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>c_doc_4cc61ecc-8ab9-4348-9905-a710c3c0e65a_JPG_1</t>
+          <t>c_doc_4cc61ecc-8ab9-4348-9905-a710c3c0e65a_JPG_0</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Fungal infection (inferred)</t>
+          <t>Pyoderma</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Nuforce Pet 200</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>1 tablet</t>
-        </is>
-      </c>
+          <t>Onyfle lotion</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr"/>
       <c r="G6" s="2" t="inlineStr"/>
       <c r="H6" s="2" t="inlineStr"/>
@@ -1765,28 +1661,28 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>c_doc_887afa02-5a78-4725-8c70-3e1c81ec7ded_JPG_0</t>
+          <t>c_doc_4cc61ecc-8ab9-4348-9905-a710c3c0e65a_JPG_0</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Post-neuter surgical care</t>
+          <t>Pyoderma</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Rivcet spray</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr"/>
+          <t>Nuforce Pet 200</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>1 tablet</t>
+        </is>
+      </c>
       <c r="F7" s="3" t="inlineStr"/>
       <c r="G7" s="3" t="inlineStr"/>
       <c r="H7" s="3" t="inlineStr"/>
-      <c r="I7" s="3" t="inlineStr">
-        <is>
-          <t>2023-02-10</t>
-        </is>
-      </c>
+      <c r="I7" s="3" t="inlineStr"/>
       <c r="J7" s="3" t="inlineStr">
         <is>
           <t>medicine</t>
@@ -1806,12 +1702,12 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Post-neuter surgical care</t>
+          <t>Post-neutering care (inferred)</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Wound Heal powder</t>
+          <t>Rivcet spray</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
@@ -1842,12 +1738,12 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Post-neuter surgical care</t>
+          <t>Post-neutering care (inferred)</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Capril 100</t>
+          <t>Wound Heal powder</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr"/>
@@ -1878,12 +1774,12 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Post-neuter surgical care</t>
+          <t>Post-neutering care (inferred)</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Cefpet CLV</t>
+          <t>Capril 100</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
@@ -1914,12 +1810,12 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Post-neuter surgical care</t>
+          <t>Post-neutering care (inferred)</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Pantopet 40</t>
+          <t>Cefpet-CLV</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr"/>
@@ -1945,30 +1841,26 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>c_doc_cb8881ad-2432-49f8-91a4-3aa752b4d4a1_JPG_0</t>
+          <t>c_doc_887afa02-5a78-4725-8c70-3e1c81ec7ded_JPG_0</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Musculoskeletal pain (inferred)</t>
+          <t>Post-neutering care (inferred)</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Carital</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>10 mg, 1/2 tablet</t>
-        </is>
-      </c>
+          <t>Pantopet 40</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr"/>
       <c r="G12" s="2" t="inlineStr"/>
       <c r="H12" s="2" t="inlineStr"/>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>2022-12-10</t>
+          <t>2023-02-10</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1995,14 +1887,22 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Hot fomentation</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr"/>
+          <t>Carital</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>10 mg, 1/2 tablet</t>
+        </is>
+      </c>
       <c r="F13" s="3" t="inlineStr"/>
       <c r="G13" s="3" t="inlineStr"/>
       <c r="H13" s="3" t="inlineStr"/>
-      <c r="I13" s="3" t="inlineStr"/>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>2022-12-10</t>
+        </is>
+      </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
           <t>medicine</t>
@@ -2133,7 +2033,7 @@
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
@@ -2184,7 +2084,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Post-neuter surgical care</t>
+          <t>Post-neutering care (inferred)</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -2212,7 +2112,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Post-neuter surgical care</t>
+          <t>Post-neutering care (inferred)</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -2270,7 +2170,7 @@
     <col width="37" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="21" customWidth="1" min="9" max="9"/>
@@ -2425,12 +2325,12 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Pyoderma (inferred)</t>
+          <t>Pyoderma</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>recurrent</t>
+          <t>episodic</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -2440,7 +2340,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>2024-12-19, 2026-05-01, 2026-05-02</t>
+          <t>2024-12-19</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -2450,7 +2350,7 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2024-12-19</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -2460,21 +2360,21 @@
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
           <t>c_doc_f4d47d0c-db22-43c6-b757-9b10adb74446_JPG_0</t>
         </is>
       </c>
       <c r="M3" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -2490,7 +2390,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Post-neuter surgical care</t>
+          <t>Post-neutering care (inferred)</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -2705,7 +2605,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Nutracillin B13</t>
+          <t>Nutrolin B</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -2719,12 +2619,12 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Pyoderma (inferred)</t>
+          <t>Pyoderma</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Onfite lotion</t>
+          <t>Betadine</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr"/>
@@ -2734,50 +2634,46 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Pyoderma (inferred)</t>
+          <t>Pyoderma</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Nuforce Pet 200</t>
+          <t>Onyfle lotion</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr"/>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>1 tablet</t>
-        </is>
-      </c>
+      <c r="D6" s="2" t="n"/>
       <c r="E6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Pyoderma (inferred)</t>
+          <t>Pyoderma</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Itraconazole</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>2024-12-29</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="n"/>
+          <t>Nuforce Pet 200</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>1 tablet</t>
+        </is>
+      </c>
       <c r="E7" s="3" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Pyoderma (inferred)</t>
+          <t>Pyoderma</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Pantoprazole+Domperidone</t>
+          <t>Itraconazole</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -2791,12 +2687,12 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Pyoderma (inferred)</t>
+          <t>Pyoderma</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Onfyte lotion</t>
+          <t>Pantoprazole+Domperidone</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -2810,17 +2706,17 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Post-neuter surgical care</t>
+          <t>Pyoderma</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Rivcet spray</t>
+          <t>Onfyte lotion</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>2023-02-10</t>
+          <t>2024-12-29</t>
         </is>
       </c>
       <c r="D10" s="2" t="n"/>
@@ -2829,12 +2725,12 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Post-neuter surgical care</t>
+          <t>Post-neutering care (inferred)</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Wound Heal powder</t>
+          <t>Rivcet spray</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -2848,12 +2744,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Post-neuter surgical care</t>
+          <t>Post-neutering care (inferred)</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Capril 100</t>
+          <t>Wound Heal powder</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -2867,12 +2763,12 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Post-neuter surgical care</t>
+          <t>Post-neutering care (inferred)</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Cefpet CLV</t>
+          <t>Capril 100</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -2886,12 +2782,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Post-neuter surgical care</t>
+          <t>Post-neutering care (inferred)</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Pantopet 40</t>
+          <t>Cefpet-CLV</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -2905,24 +2801,20 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Musculoskeletal pain (inferred)</t>
+          <t>Post-neutering care (inferred)</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Carital</t>
+          <t>Pantopet 40</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>2022-12-10</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>10 mg, 1/2 tablet</t>
-        </is>
-      </c>
+          <t>2023-02-10</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="n"/>
       <c r="E15" s="3" t="n"/>
     </row>
     <row r="16">
@@ -2933,11 +2825,19 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Hot fomentation</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr"/>
-      <c r="D16" s="2" t="n"/>
+          <t>Carital</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>2022-12-10</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>10 mg, 1/2 tablet</t>
+        </is>
+      </c>
       <c r="E16" s="2" t="n"/>
     </row>
   </sheetData>

</xml_diff>